<commit_message>
Log template changes not saved previously...
</commit_message>
<xml_diff>
--- a/log_templates/OBS Deployment Summary Template.xlsx
+++ b/log_templates/OBS Deployment Summary Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dalu-my.sharepoint.com/personal/kt679536_dal_ca/Documents/NFSI/Projects/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Katie Bosman\code\OBSDataPipeline\log_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="221" documentId="8_{06774BE9-7577-4792-9C8B-B53C3A141BAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC0F6D48-DF5D-44FB-8267-F8CFD3BCAA42}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7A4C26-23EF-402C-B993-F69B99E2C167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-4512" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{40123D5C-8A56-48C8-83AB-25C6150FC8B9}"/>
+    <workbookView xWindow="-38510" yWindow="-10910" windowWidth="38620" windowHeight="21220" xr2:uid="{40123D5C-8A56-48C8-83AB-25C6150FC8B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="57">
   <si>
     <t>Station Name</t>
   </si>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>Dunker</t>
+  </si>
+  <si>
+    <t>Released</t>
   </si>
 </sst>
 </file>
@@ -599,34 +602,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D05B9B89-AA38-4C80-A270-6884D62EF09D}">
-  <dimension ref="A1:AB14"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.85546875" customWidth="1"/>
+    <col min="20" max="20" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="26.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -640,39 +645,42 @@
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
       <c r="N1" s="6"/>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
       <c r="R1" s="6"/>
       <c r="S1" s="6"/>
       <c r="T1" s="6"/>
       <c r="U1" s="6"/>
-      <c r="V1" s="6" t="s">
-        <v>24</v>
-      </c>
+      <c r="V1" s="6"/>
       <c r="W1" s="6"/>
       <c r="X1" s="6"/>
-      <c r="Y1" s="6"/>
-      <c r="Z1" s="6" t="s">
-        <v>38</v>
-      </c>
+      <c r="Y1" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="6"/>
       <c r="AA1" s="6"/>
       <c r="AB1" s="6"/>
-    </row>
-    <row r="2" spans="1:28" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="AC1" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD1" s="6"/>
+      <c r="AE1" s="6"/>
+    </row>
+    <row r="2" spans="1:31" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>7</v>
       </c>
@@ -683,159 +691,168 @@
         <v>42</v>
       </c>
       <c r="E2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="J2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="S2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="T2" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="X2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="Y2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="Z2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="AA2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="AB2" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="AC2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AD2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AE2" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N3" s="2">
-        <f t="shared" ref="N3" si="0">2*6370*ASIN(SQRT(SIN(RADIANS(K3-H3)/2)*SIN(RADIANS(K3-H3)/2) + COS(RADIANS(K3))*COS(RADIANS(H3))*SIN(RADIANS(L3-I3)/2)*SIN(RADIANS(L3-I3)/2)))</f>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P3" s="2">
+        <f t="shared" ref="P3" si="0">2*6370*ASIN(SQRT(SIN(RADIANS(M3-J3)/2)*SIN(RADIANS(M3-J3)/2) + COS(RADIANS(M3))*COS(RADIANS(J3))*SIN(RADIANS(N3-K3)/2)*SIN(RADIANS(N3-K3)/2)))</f>
         <v>0</v>
       </c>
-      <c r="T3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(O3-K3)/2)*SIN(RADIANS(O3-K3)/2) + COS(RADIANS(O3))*COS(RADIANS(K3))*SIN(RADIANS(P3-L3)/2)*SIN(RADIANS(P3-L3)/2)))*1000</f>
+      <c r="W3" s="2">
+        <f>2*6370*ASIN(SQRT(SIN(RADIANS(Q3-M3)/2)*SIN(RADIANS(Q3-M3)/2) + COS(RADIANS(Q3))*COS(RADIANS(M3))*SIN(RADIANS(R3-N3)/2)*SIN(RADIANS(R3-N3)/2)))*1000</f>
         <v>0</v>
       </c>
-      <c r="U3" t="e">
-        <f>MOD(DEGREES(ATAN2(COS(RADIANS(K3))*SIN(RADIANS(O3)) - SIN(RADIANS(K3))*COS(RADIANS(O3))*COS(RADIANS(P3-L3)),COS(RADIANS(O3))*SIN(RADIANS(P3-L3)))) + 360, 360)</f>
+      <c r="X3" t="e">
+        <f>MOD(DEGREES(ATAN2(COS(RADIANS(M3))*SIN(RADIANS(Q3)) - SIN(RADIANS(M3))*COS(RADIANS(Q3))*COS(RADIANS(R3-N3)),COS(RADIANS(Q3))*SIN(RADIANS(R3-N3)))) + 360, 360)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="X3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(V3-O3)/2)*SIN(RADIANS(V3-O3)/2) + COS(RADIANS(V3))*COS(RADIANS(O3))*SIN(RADIANS(W3-P3)/2)*SIN(RADIANS(W3-P3)/2)))*1000</f>
+      <c r="AA3" s="2">
+        <f>2*6370*ASIN(SQRT(SIN(RADIANS(Y3-Q3)/2)*SIN(RADIANS(Y3-Q3)/2) + COS(RADIANS(Y3))*COS(RADIANS(Q3))*SIN(RADIANS(Z3-R3)/2)*SIN(RADIANS(Z3-R3)/2)))*1000</f>
         <v>0</v>
       </c>
-      <c r="Y3" t="e">
-        <f>MOD(DEGREES(ATAN2(COS(RADIANS(O3))*SIN(RADIANS(V3)) - SIN(RADIANS(O3))*COS(RADIANS(V3))*COS(RADIANS(W3-P3)),COS(RADIANS(V3))*SIN(RADIANS(W3-P3)))) + 360, 360)</f>
+      <c r="AB3" t="e">
+        <f>MOD(DEGREES(ATAN2(COS(RADIANS(Q3))*SIN(RADIANS(Y3)) - SIN(RADIANS(Q3))*COS(RADIANS(Y3))*COS(RADIANS(Z3-R3)),COS(RADIANS(Y3))*SIN(RADIANS(Z3-R3)))) + 360, 360)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AB3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(Z3-V3)/2)*SIN(RADIANS(Z3-V3)/2) + COS(RADIANS(Z3))*COS(RADIANS(V3))*SIN(RADIANS(AA3-X3)/2)*SIN(RADIANS(AA3-X3)/2)))</f>
+      <c r="AE3" s="2">
+        <f>2*6370*ASIN(SQRT(SIN(RADIANS(AC3-Y3)/2)*SIN(RADIANS(AC3-Y3)/2) + COS(RADIANS(AC3))*COS(RADIANS(Y3))*SIN(RADIANS(AD3-AA3)/2)*SIN(RADIANS(AD3-AA3)/2)))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N4" s="2"/>
-      <c r="T4" s="2"/>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N5" s="2"/>
-      <c r="T5" s="2"/>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N6" s="2"/>
-      <c r="T6" s="2"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N7" s="2"/>
-      <c r="T7" s="2"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N8" s="2"/>
-      <c r="T8" s="2"/>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N9" s="2"/>
-      <c r="T9" s="2"/>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N10" s="2"/>
-      <c r="T10" s="2"/>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N11" s="2"/>
-      <c r="T11" s="2"/>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N12" s="2"/>
-      <c r="T12" s="2"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N13" s="2"/>
-      <c r="T13" s="2"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="N14" s="2"/>
-      <c r="T14" s="2"/>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P4" s="2"/>
+      <c r="W4" s="2"/>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P5" s="2"/>
+      <c r="W5" s="2"/>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P6" s="2"/>
+      <c r="W6" s="2"/>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P7" s="2"/>
+      <c r="W7" s="2"/>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P8" s="2"/>
+      <c r="W8" s="2"/>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P9" s="2"/>
+      <c r="W9" s="2"/>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P10" s="2"/>
+      <c r="W10" s="2"/>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P11" s="2"/>
+      <c r="W11" s="2"/>
+    </row>
+    <row r="12" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P12" s="2"/>
+      <c r="W12" s="2"/>
+    </row>
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P13" s="2"/>
+      <c r="W13" s="2"/>
+    </row>
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="P14" s="2"/>
+      <c r="W14" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="Z1:AB1"/>
-    <mergeCell ref="O1:U1"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="AC1:AE1"/>
+    <mergeCell ref="Q1:X1"/>
+    <mergeCell ref="J1:L1"/>
+    <mergeCell ref="M1:P1"/>
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="V1:Y1"/>
-    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="Y1:AB1"/>
+    <mergeCell ref="D1:I1"/>
   </mergeCells>
-  <conditionalFormatting sqref="N3:N14">
+  <conditionalFormatting sqref="P3:P14">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -847,7 +864,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T3:T14">
+  <conditionalFormatting sqref="W3:W14">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -859,7 +876,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X3">
+  <conditionalFormatting sqref="AA3">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -871,7 +888,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB3">
+  <conditionalFormatting sqref="AE3">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1172,27 +1189,28 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90C860AB-45FF-4001-B438-BC557F0592A0}">
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:X3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="9.140625" customWidth="1"/>
-    <col min="12" max="12" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" customWidth="1"/>
-    <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" customWidth="1"/>
-    <col min="17" max="17" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="100.5703125" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="100.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1215,31 +1233,32 @@
       <c r="J1" s="6"/>
       <c r="K1" s="6"/>
       <c r="L1" s="6"/>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="6"/>
+      <c r="N1" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="N1" s="6"/>
       <c r="O1" s="6"/>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="Q1" s="6"/>
       <c r="R1" s="6"/>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="6"/>
+      <c r="T1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="T1" s="6"/>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="6"/>
+      <c r="V1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:23" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1265,49 +1284,52 @@
         <v>33</v>
       </c>
       <c r="J2" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="N2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="O2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="P2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="Q2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="R2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="S2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="O3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(M3-B3)/2)*SIN(RADIANS(M3-B3)/2) + COS(RADIANS(M3))*COS(RADIANS(B3))*SIN(RADIANS(N3-C3)/2)*SIN(RADIANS(N3-C3)/2)))</f>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="P3" s="2">
+        <f>2*6370*ASIN(SQRT(SIN(RADIANS(N3-B3)/2)*SIN(RADIANS(N3-B3)/2) + COS(RADIANS(N3))*COS(RADIANS(B3))*SIN(RADIANS(O3-C3)/2)*SIN(RADIANS(O3-C3)/2)))</f>
         <v>0</v>
       </c>
-      <c r="R3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(P3-M3)/2)*SIN(RADIANS(P3-M3)/2) + COS(RADIANS(P3))*COS(RADIANS(M3))*SIN(RADIANS(Q3-N3)/2)*SIN(RADIANS(Q3-N3)/2)))</f>
+      <c r="S3" s="2">
+        <f>2*6370*ASIN(SQRT(SIN(RADIANS(Q3-N3)/2)*SIN(RADIANS(Q3-N3)/2) + COS(RADIANS(Q3))*COS(RADIANS(N3))*SIN(RADIANS(R3-O3)/2)*SIN(RADIANS(R3-O3)/2)))</f>
         <v>0</v>
       </c>
     </row>
@@ -1316,12 +1338,12 @@
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="G1:H1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="P1:R1"/>
-    <mergeCell ref="I1:L1"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="T1:U1"/>
+    <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="I1:M1"/>
   </mergeCells>
-  <conditionalFormatting sqref="O3">
+  <conditionalFormatting sqref="P3">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1333,7 +1355,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R3">
+  <conditionalFormatting sqref="S3">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>